<commit_message>
feat: add 4 bank profiles for ABA and Acleda, fix 26-Oct-26 date parsing and shifted row detection
</commit_message>
<xml_diff>
--- a/Account id aba.xlsx
+++ b/Account id aba.xlsx
@@ -47,22 +47,22 @@
     <t>001 746 626</t>
   </si>
   <si>
-    <t>C00169</t>
+    <t>C02036</t>
   </si>
   <si>
-    <t>nana</t>
+    <t>M25 Dental Clinic</t>
   </si>
   <si>
-    <t>096 441 100</t>
+    <t>000598739</t>
   </si>
   <si>
-    <t>C00170</t>
+    <t>C01898</t>
   </si>
   <si>
-    <t>keke</t>
+    <t>PAID BY IM DAREN</t>
   </si>
   <si>
-    <t>000 755 553</t>
+    <t>34480658932428</t>
   </si>
 </sst>
 </file>
@@ -698,7 +698,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -708,6 +708,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1237,6 +1244,7 @@
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="3" width="22.2857142857143" customWidth="1"/>
+    <col min="4" max="4" width="14.3904761904762" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1268,7 +1276,7 @@
       <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="6" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1279,7 +1287,7 @@
       <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="7" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: auto-allocate ABA payments to newest invoices and allow interactive checkbox settlement with payment ceiling
</commit_message>
<xml_diff>
--- a/Account id aba.xlsx
+++ b/Account id aba.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Entry No</t>
   </si>
@@ -50,7 +50,14 @@
     <t>C02036</t>
   </si>
   <si>
-    <t>M25 Dental Clinic</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>M25 Dental Clinic</t>
+    </r>
   </si>
   <si>
     <t>000598739</t>
@@ -63,6 +70,15 @@
   </si>
   <si>
     <t>34480658932428</t>
+  </si>
+  <si>
+    <t>C00045</t>
+  </si>
+  <si>
+    <t>Beauty Smile Dental Clinic</t>
+  </si>
+  <si>
+    <t>025934450001/001 654 720</t>
   </si>
 </sst>
 </file>
@@ -75,7 +91,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,6 +102,11 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Khmer OS Moul"/>
       <charset val="134"/>
     </font>
     <font>
@@ -568,137 +589,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -708,12 +729,19 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" quotePrefix="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1240,10 +1268,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="2"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="2"/>
   <cols>
-    <col min="1" max="3" width="22.2857142857143" customWidth="1"/>
+    <col min="1" max="1" width="22.2857142857143" customWidth="1"/>
+    <col min="2" max="2" width="29.3333333333333" customWidth="1"/>
+    <col min="3" max="3" width="30.3333333333333" customWidth="1"/>
     <col min="4" max="4" width="14.3904761904762" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1273,10 +1303,10 @@
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="8" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1287,9 +1317,24 @@
       <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="9" t="s">
         <v>11</v>
       </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="7"/>
+      <c r="B6" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(reconciliation): save uploads strictly in uploads subfolder, clear server cache on upload, preserve Drive H on reset, purge Ong Mach
</commit_message>
<xml_diff>
--- a/Account id aba.xlsx
+++ b/Account id aba.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Entry No</t>
   </si>
@@ -36,49 +36,6 @@
   </si>
   <si>
     <t>accound aba</t>
-  </si>
-  <si>
-    <t>C00168</t>
-  </si>
-  <si>
-    <t>Ong Mach</t>
-  </si>
-  <si>
-    <t>001 746 626</t>
-  </si>
-  <si>
-    <t>C02036</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>M25 Dental Clinic</t>
-    </r>
-  </si>
-  <si>
-    <t>000598739</t>
-  </si>
-  <si>
-    <t>C01898</t>
-  </si>
-  <si>
-    <t>PAID BY IM DAREN</t>
-  </si>
-  <si>
-    <t>34480658932428</t>
-  </si>
-  <si>
-    <t>C00045</t>
-  </si>
-  <si>
-    <t>Beauty Smile Dental Clinic</t>
-  </si>
-  <si>
-    <t>025934450001/001 654 720</t>
   </si>
 </sst>
 </file>
@@ -734,13 +691,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" quotePrefix="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1289,48 +1239,24 @@
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>5</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>8</v>
-      </c>
+    <row r="3" ht="23.25" spans="1:3">
+      <c r="A3" s="4"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="2"/>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>11</v>
-      </c>
+      <c r="A4" s="4"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="6"/>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>14</v>
-      </c>
+      <c r="A5" s="7"/>
+      <c r="B5" s="7"/>
+      <c r="C5" s="7"/>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="7"/>

</xml_diff>